<commit_message>
Fix OpenXML schema-validity bugs in Word and Excel output
Fix OpenXML schema-validity bugs in Word and Excel output

All produced documents that Word/Excel flag as corrupt on open; none were
caught because the Verify snapshots never ran OpenXmlValidator.

- Word rPr: emit children in CT_RPr order (rFonts, b, color, sz, szCs, u)
- Word standalone tblBorders: order top, left, bottom, right, insideH, insideV
- Excel worksheet: place conditionalFormatting/dataValidations before <hyperlinks>
- Excel font/fill rgb: write 8-digit ARGB and emit <color> before <name> in
  CT_Font; fixes every linked workbook and any 6-digit user color. List-link
  inline runs now order color before u.

Add OpenXmlValidator coverage for each path; re-verify affected snapshots.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/LinkTests.Null.verified.xlsx
+++ b/src/Excelsior.Tests/LinkTests.Null.verified.xlsx
@@ -22,8 +22,8 @@
     <font>
       <u/>
       <sz val="11"/>
+      <color rgb="FF0563C1"/>
       <name val="Calibri"/>
-      <color rgb="0563C1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -121,8 +121,8 @@
           </r>
           <r>
             <rPr>
+              <color rgb="FF0563C1"/>
               <u/>
-              <color rgb="0563C1"/>
             </rPr>
             <t xml:space="preserve">Google (https://google.com)</t>
           </r>

</xml_diff>

<commit_message>
Fix OpenXML schema-validity bugs in Word and Excel output (#238)
Fix OpenXML schema-validity bugs in Word and Excel output

All produced documents that Word/Excel flag as corrupt on open; none were
caught because the Verify snapshots never ran OpenXmlValidator.

- Word rPr: emit children in CT_RPr order (rFonts, b, color, sz, szCs, u)
- Word standalone tblBorders: order top, left, bottom, right, insideH, insideV
- Excel worksheet: place conditionalFormatting/dataValidations before <hyperlinks>
- Excel font/fill rgb: write 8-digit ARGB and emit <color> before <name> in
  CT_Font; fixes every linked workbook and any 6-digit user color. List-link
  inline runs now order color before u.

Add OpenXmlValidator coverage for each path; re-verify affected snapshots.
</commit_message>
<xml_diff>
--- a/src/Excelsior.Tests/LinkTests.Null.verified.xlsx
+++ b/src/Excelsior.Tests/LinkTests.Null.verified.xlsx
@@ -22,8 +22,8 @@
     <font>
       <u/>
       <sz val="11"/>
+      <color rgb="FF0563C1"/>
       <name val="Calibri"/>
-      <color rgb="0563C1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -121,8 +121,8 @@
           </r>
           <r>
             <rPr>
+              <color rgb="FF0563C1"/>
               <u/>
-              <color rgb="0563C1"/>
             </rPr>
             <t xml:space="preserve">Google (https://google.com)</t>
           </r>

</xml_diff>